<commit_message>
polish dashboard warning states
</commit_message>
<xml_diff>
--- a/backtest.xlsx
+++ b/backtest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="backtest" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="settled_only" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="backtest" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settled_only" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,117 +430,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>平台</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>比赛时间</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>比赛时间(北京时间)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>记录日期(北京时间)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>发现时间UTC</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>开赛快照时间UTC</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>开赛主队概率</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>开赛客队概率</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>主队</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>客队</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>主队概率</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>客队概率</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>赔率</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>预测嬴方</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>实际嬴方（后续补充）</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>跨市场主队价差</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>跨市场客队价差</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>价差预警</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>是否命中</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>下注方向</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>10U收益</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>累计收益</t>
         </is>
@@ -929,7 +941,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-03-29T13:59:58.648921+00:00</t>
+          <t>2026-03-29T14:33:57.207446+00:00</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1008,7 +1020,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-03-29T13:59:58.371452+00:00</t>
+          <t>2026-03-29T14:33:55.654097+00:00</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1087,7 +1099,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-03-29T13:59:58.779000+00:00</t>
+          <t>2026-03-29T14:33:58.731002+00:00</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1109,14 +1121,14 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>0.205</v>
+        <v>0.225</v>
       </c>
       <c r="M8" t="n">
-        <v>0.795</v>
+        <v>0.785</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Indiana Pacers 0.205 | Miami Heat 0.795</t>
+          <t>Indiana Pacers 0.225 | Miami Heat 0.785</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1166,7 +1178,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-03-29T13:59:58.372611+00:00</t>
+          <t>2026-03-29T14:33:55.654097+00:00</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1188,14 +1200,14 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
       <c r="M9" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Indiana Pacers 0.210 | Miami Heat 0.800</t>
+          <t>Indiana Pacers 0.220 | Miami Heat 0.790</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1245,7 +1257,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-03-29T13:59:59.009696+00:00</t>
+          <t>2026-03-29T14:34:00.231475+00:00</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1267,14 +1279,14 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>0.495</v>
+        <v>0.49</v>
       </c>
       <c r="M10" t="n">
-        <v>0.505</v>
+        <v>0.515</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Brooklyn Nets 0.495 | Sacramento Kings 0.505</t>
+          <t>Brooklyn Nets 0.490 | Sacramento Kings 0.515</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1284,7 +1296,7 @@
       </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
         <v>0.005</v>
@@ -1324,7 +1336,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-03-29T13:59:59.097790+00:00</t>
+          <t>2026-03-29T14:34:02.711491+00:00</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1403,7 +1415,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-03-29T13:59:59.486316+00:00</t>
+          <t>2026-03-29T14:34:05.656783+00:00</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1478,7 +1490,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-03-29T13:59:59.326721+00:00</t>
+          <t>2026-03-29T14:34:04.123138+00:00</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1500,14 +1512,14 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>0.555</v>
+        <v>0.545</v>
       </c>
       <c r="M13" t="n">
         <v>0.455</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Toronto Raptors 0.555 | Orlando Magic 0.455</t>
+          <t>Toronto Raptors 0.545 | Orlando Magic 0.455</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1517,7 +1529,7 @@
       </c>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="n">
-        <v>0.005</v>
+        <v>0.015</v>
       </c>
       <c r="R13" t="n">
         <v>0.015</v>
@@ -1557,7 +1569,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-03-29T13:06:27.205454+00:00</t>
+          <t>2026-03-29T14:33:55.659334+00:00</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1579,14 +1591,14 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
       <c r="M14" t="n">
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Brooklyn Nets 0.500 | Sacramento Kings 0.510</t>
+          <t>Brooklyn Nets 0.490 | Sacramento Kings 0.520</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1596,7 +1608,7 @@
       </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="R14" t="n">
         <v>0.005</v>
@@ -1636,7 +1648,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-03-29T13:59:58.371284+00:00</t>
+          <t>2026-03-29T14:33:55.651705+00:00</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1754,7 +1766,7 @@
       </c>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="n">
-        <v>0.005</v>
+        <v>0.015</v>
       </c>
       <c r="R16" t="n">
         <v>0.015</v>
@@ -1794,7 +1806,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-03-29T13:59:58.372844+00:00</t>
+          <t>2026-03-29T14:33:55.654097+00:00</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1944,7 +1956,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-03-29T13:59:59.910466+00:00</t>
+          <t>2026-03-29T14:34:11.758681+00:00</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1969,11 +1981,11 @@
         <v>0.5</v>
       </c>
       <c r="M19" t="n">
-        <v>0.49</v>
+        <v>0.495</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Miami Heat 0.500 | Philadelphia 76ers 0.490</t>
+          <t>Miami Heat 0.500 | Philadelphia 76ers 0.495</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -2019,7 +2031,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-03-29T14:00:00.007851+00:00</t>
+          <t>2026-03-29T14:34:13.499336+00:00</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2094,7 +2106,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-03-29T13:59:58.377538+00:00</t>
+          <t>2026-03-29T14:33:55.660335+00:00</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2244,7 +2256,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-03-29T13:59:58.377228+00:00</t>
+          <t>2026-03-29T14:33:55.659334+00:00</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2266,14 +2278,14 @@
         </is>
       </c>
       <c r="L23" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="M23" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Los Angeles Lakers 0.920 | Washington Wizards 0.090</t>
+          <t>Los Angeles Lakers 0.930 | Washington Wizards 0.080</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -2319,7 +2331,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-03-29T14:00:00.801297+00:00</t>
+          <t>2026-03-29T14:34:25.738354+00:00</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2341,14 +2353,14 @@
         </is>
       </c>
       <c r="L24" t="n">
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
       <c r="M24" t="n">
         <v>0.455</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Orlando Magic 0.380 | Phoenix Suns 0.455</t>
+          <t>Orlando Magic 0.360 | Phoenix Suns 0.455</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -2386,117 +2398,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>平台</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>比赛时间</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>比赛时间(北京时间)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>记录日期(北京时间)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>发现时间UTC</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>开赛快照时间UTC</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>开赛主队概率</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>开赛客队概率</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>主队</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>客队</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>主队概率</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>客队概率</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>赔率</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>预测嬴方</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>实际嬴方（后续补充）</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>跨市场主队价差</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>跨市场客队价差</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>价差预警</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>是否命中</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>下注方向</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>10U收益</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>累计收益</t>
         </is>

</xml_diff>

<commit_message>
enhance sportsbook comparison dashboard
</commit_message>
<xml_diff>
--- a/backtest.xlsx
+++ b/backtest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="backtest" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="settled_only" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="backtest" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settled_only" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,152 +430,152 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>平台</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>比赛时间</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>比赛时间(北京时间)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>记录日期(北京时间)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>发现时间UTC</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>开赛快照时间UTC</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>开赛主队概率</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>开赛客队概率</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>主流博彩主队概率</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>主流博彩客队概率</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>主流博彩样本数</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>主流博彩来源</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>主流博彩状态</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>主队</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>客队</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>主队概率</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>客队概率</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>赔率</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>预测嬴方</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>实际嬴方（后续补充）</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>跨市场主队价差</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>跨市场客队价差</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>价差预警</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>相对主流博彩主队价差</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>相对主流博彩客队价差</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>是否命中</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>下注方向</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>10U收益</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>累计收益</t>
         </is>
@@ -2814,7 +2826,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-03-30T14:39:11.862488+00:00</t>
+          <t>2026-03-30T14:55:44.070805+00:00</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2906,7 +2918,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-03-30T14:39:11.729777+00:00</t>
+          <t>2026-03-30T14:55:40.363511+00:00</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2998,7 +3010,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-03-30T14:39:12.067898+00:00</t>
+          <t>2026-03-30T14:55:46.745356+00:00</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -3182,7 +3194,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-03-30T14:39:11.732301+00:00</t>
+          <t>2026-03-30T14:55:40.369179+00:00</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3346,7 +3358,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-03-30T14:39:11.732085+00:00</t>
+          <t>2026-03-30T14:55:40.369179+00:00</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3428,7 +3440,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-03-30T14:39:11.733571+00:00</t>
+          <t>2026-03-30T14:55:40.369179+00:00</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3674,7 +3686,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-03-30T14:39:12.577518+00:00</t>
+          <t>2026-03-30T14:56:05.987867+00:00</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3760,7 +3772,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-03-30T14:39:11.735883+00:00</t>
+          <t>2026-03-30T14:55:40.381613+00:00</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3846,7 +3858,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-03-30T14:39:12.686840+00:00</t>
+          <t>2026-03-30T14:56:08.554981+00:00</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3876,11 +3888,11 @@
         <v>0.095</v>
       </c>
       <c r="R33" t="n">
-        <v>0.91</v>
+        <v>0.905</v>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>Brooklyn Nets 0.095 | Charlotte Hornets 0.910</t>
+          <t>Brooklyn Nets 0.095 | Charlotte Hornets 0.905</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -3893,7 +3905,7 @@
         <v>0.005</v>
       </c>
       <c r="W33" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="X33" t="inlineStr"/>
       <c r="Y33" t="inlineStr"/>
@@ -3932,7 +3944,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-03-30T14:39:11.735597+00:00</t>
+          <t>2026-03-30T14:55:40.381613+00:00</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3979,7 +3991,7 @@
         <v>0.005</v>
       </c>
       <c r="W34" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="X34" t="inlineStr"/>
       <c r="Y34" t="inlineStr"/>
@@ -4018,7 +4030,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-03-30T14:39:11.734881+00:00</t>
+          <t>2026-03-30T14:55:40.379582+00:00</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4100,7 +4112,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-03-30T14:39:11.735262+00:00</t>
+          <t>2026-03-30T14:55:40.379582+00:00</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4182,7 +4194,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-03-30T14:39:13.287621+00:00</t>
+          <t>2026-03-30T14:56:26.450697+00:00</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4209,14 +4221,14 @@
         </is>
       </c>
       <c r="Q37" t="n">
-        <v>0.305</v>
+        <v>0.31</v>
       </c>
       <c r="R37" t="n">
-        <v>0.375</v>
+        <v>0.395</v>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Orlando Magic 0.305 | Atlanta Hawks 0.375</t>
+          <t>Orlando Magic 0.310 | Atlanta Hawks 0.395</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
@@ -4264,7 +4276,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-03-30T14:39:13.229799+00:00</t>
+          <t>2026-03-30T14:56:22.836866+00:00</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4294,11 +4306,11 @@
         <v>0.135</v>
       </c>
       <c r="R38" t="n">
-        <v>0.845</v>
+        <v>0.85</v>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>Washington Wizards 0.135 | Philadelphia 76ers 0.845</t>
+          <t>Washington Wizards 0.135 | Philadelphia 76ers 0.850</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
@@ -4338,152 +4350,152 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>平台</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>比赛时间</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>比赛时间(北京时间)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>记录日期(北京时间)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>发现时间UTC</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>开赛快照时间UTC</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>开赛主队概率</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>开赛客队概率</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>主流博彩主队概率</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>主流博彩客队概率</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>主流博彩样本数</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>主流博彩来源</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>主流博彩状态</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>主队</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>客队</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>主队概率</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>客队概率</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>赔率</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>预测嬴方</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>实际嬴方（后续补充）</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>跨市场主队价差</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>跨市场客队价差</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>价差预警</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>相对主流博彩主队价差</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>相对主流博彩客队价差</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>是否命中</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>下注方向</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>10U收益</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>累计收益</t>
         </is>

</xml_diff>

<commit_message>
add probability bin accuracy table
</commit_message>
<xml_diff>
--- a/backtest.xlsx
+++ b/backtest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="backtest" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="settled_only" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="backtest" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settled_only" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,162 +430,162 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>平台</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>比赛时间</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>比赛时间(北京时间)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>记录日期(北京时间)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>发现时间UTC</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>开赛快照时间UTC</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>开赛主队概率</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>开赛客队概率</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>开赛主流博彩主队概率</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>开赛主流博彩客队概率</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>主流博彩主队概率</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>主流博彩客队概率</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>主流博彩样本数</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>主流博彩来源</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>主流博彩状态</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>主队</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>客队</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>主队概率</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>客队概率</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>赔率</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>预测嬴方</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>实际嬴方（后续补充）</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>跨市场主队价差</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>跨市场客队价差</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>价差预警</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>相对主流博彩主队价差</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>相对主流博彩客队价差</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>是否命中</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>下注方向</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>10U收益</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>累计收益</t>
         </is>
@@ -4078,7 +4090,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-03-31T09:47:40.618563+00:00</t>
+          <t>2026-03-31T09:50:09.652905+00:00</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -4260,7 +4272,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-03-31T09:47:40.709479+00:00</t>
+          <t>2026-03-31T09:50:11.512903+00:00</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -4526,7 +4538,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-03-31T09:47:32.798856+00:00</t>
+          <t>2026-03-31T09:49:44.982710+00:00</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4610,7 +4622,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-03-31T09:47:32.801178+00:00</t>
+          <t>2026-03-31T09:49:44.988829+00:00</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4862,7 +4874,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-03-31T09:47:41.323593+00:00</t>
+          <t>2026-03-31T09:50:24.874600+00:00</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4946,7 +4958,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-03-31T09:47:41.238976+00:00</t>
+          <t>2026-03-31T09:50:22.817131+00:00</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -5030,7 +5042,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-03-31T09:47:41.411917+00:00</t>
+          <t>2026-03-31T09:50:26.722943+00:00</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -5114,7 +5126,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-03-31T09:47:32.802034+00:00</t>
+          <t>2026-03-31T09:49:44.989338+00:00</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -5198,7 +5210,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-03-31T09:47:32.801639+00:00</t>
+          <t>2026-03-31T09:49:44.989338+00:00</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -5274,162 +5286,162 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>平台</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>比赛时间</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>比赛时间(北京时间)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>记录日期(北京时间)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>发现时间UTC</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>开赛快照时间UTC</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>开赛主队概率</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>开赛客队概率</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>开赛主流博彩主队概率</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>开赛主流博彩客队概率</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>主流博彩主队概率</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>主流博彩客队概率</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>主流博彩样本数</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>主流博彩来源</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>主流博彩状态</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>主队</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>客队</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>主队概率</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>客队概率</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>赔率</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>预测嬴方</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>实际嬴方（后续补充）</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>跨市场主队价差</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>跨市场客队价差</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>价差预警</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>相对主流博彩主队价差</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>相对主流博彩客队价差</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>是否命中</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>下注方向</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>10U收益</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>累计收益</t>
         </is>

</xml_diff>

<commit_message>
Fix settle logic to use stored results first
</commit_message>
<xml_diff>
--- a/backtest.xlsx
+++ b/backtest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="backtest" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="settled_only" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="backtest" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settled_only" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -582,7 +582,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -958,7 +958,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1888,7 +1888,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3092,7 +3092,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3288,7 +3288,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3586,7 +3586,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3790,7 +3790,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3892,7 +3892,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3990,7 +3990,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -4088,7 +4088,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4186,7 +4186,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -4288,7 +4288,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4390,7 +4390,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4492,7 +4492,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -4696,7 +4696,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -4802,7 +4802,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -4904,7 +4904,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -5174,7 +5174,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -5258,7 +5258,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -5342,7 +5342,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5444,7 +5444,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5538,7 +5538,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -5644,7 +5644,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -5750,7 +5750,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -5856,7 +5856,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -5962,7 +5962,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -6166,7 +6166,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -6268,7 +6268,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -6370,7 +6370,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -6476,7 +6476,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -6688,7 +6688,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -6798,7 +6798,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -6900,7 +6900,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -7100,7 +7100,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -7202,7 +7202,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -7304,7 +7304,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -7406,7 +7406,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
@@ -7490,7 +7490,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -7584,7 +7584,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -7690,7 +7690,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -7788,7 +7788,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -7894,7 +7894,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -7996,7 +7996,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8098,7 +8098,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -8202,7 +8202,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -8306,7 +8306,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -8406,7 +8406,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -8510,7 +8510,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -8818,7 +8818,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -9026,7 +9026,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -9130,7 +9130,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -9230,7 +9230,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -9330,7 +9330,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -9426,7 +9426,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -9522,7 +9522,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -9626,7 +9626,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -9730,7 +9730,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -9810,7 +9810,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -9898,7 +9898,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -9970,7 +9970,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -10114,7 +10114,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -10198,7 +10198,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -10270,7 +10270,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -10426,7 +10426,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -10498,7 +10498,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -10570,7 +10570,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -10642,7 +10642,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -10714,7 +10714,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -10782,7 +10782,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -10850,7 +10850,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
@@ -10922,7 +10922,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
@@ -10994,7 +10994,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
@@ -11066,7 +11066,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
@@ -11138,7 +11138,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
@@ -11210,7 +11210,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
@@ -11282,7 +11282,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -11354,7 +11354,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -11426,7 +11426,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -11570,7 +11570,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -11642,7 +11642,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -11714,7 +11714,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
@@ -11786,7 +11786,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F121" t="inlineStr"/>
@@ -11858,7 +11858,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
@@ -11930,7 +11930,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F123" t="inlineStr"/>
@@ -12002,7 +12002,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
@@ -12074,7 +12074,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -12146,7 +12146,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -12218,7 +12218,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
@@ -12286,7 +12286,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F128" t="inlineStr"/>
@@ -12358,7 +12358,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F129" t="inlineStr"/>
@@ -12426,7 +12426,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
@@ -12494,7 +12494,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F131" t="inlineStr"/>
@@ -12562,7 +12562,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F132" t="inlineStr"/>
@@ -12630,7 +12630,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F133" t="inlineStr"/>
@@ -12698,7 +12698,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F134" t="inlineStr"/>
@@ -12766,7 +12766,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F135" t="inlineStr"/>
@@ -12838,7 +12838,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F136" t="inlineStr"/>
@@ -12910,7 +12910,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F137" t="inlineStr"/>
@@ -12982,7 +12982,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F138" t="inlineStr"/>
@@ -13054,7 +13054,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
@@ -13126,7 +13126,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F140" t="inlineStr"/>
@@ -13198,7 +13198,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F141" t="inlineStr"/>
@@ -13270,7 +13270,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F142" t="inlineStr"/>
@@ -13342,7 +13342,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F143" t="inlineStr"/>
@@ -13414,7 +13414,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F144" t="inlineStr"/>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F145" t="inlineStr"/>
@@ -13558,7 +13558,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F146" t="inlineStr"/>
@@ -13626,7 +13626,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F147" t="inlineStr"/>
@@ -13694,7 +13694,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F148" t="inlineStr"/>
@@ -13766,7 +13766,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F149" t="inlineStr"/>
@@ -13838,7 +13838,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F150" t="inlineStr"/>
@@ -13910,7 +13910,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F151" t="inlineStr"/>
@@ -13982,7 +13982,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F152" t="inlineStr"/>
@@ -14054,7 +14054,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F153" t="inlineStr"/>
@@ -14126,7 +14126,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F154" t="inlineStr"/>
@@ -14198,7 +14198,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F155" t="inlineStr"/>
@@ -14340,12 +14340,8 @@
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr"/>
-      <c r="I157" t="n">
-        <v>0.4396</v>
-      </c>
-      <c r="J157" t="n">
-        <v>0.5604</v>
-      </c>
+      <c r="I157" t="inlineStr"/>
+      <c r="J157" t="inlineStr"/>
       <c r="K157" t="inlineStr">
         <is>
           <t>Atlanta Hawks</t>
@@ -14408,12 +14404,8 @@
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr"/>
       <c r="H158" t="inlineStr"/>
-      <c r="I158" t="n">
-        <v>0.3212</v>
-      </c>
-      <c r="J158" t="n">
-        <v>0.6788</v>
-      </c>
+      <c r="I158" t="inlineStr"/>
+      <c r="J158" t="inlineStr"/>
       <c r="K158" t="inlineStr">
         <is>
           <t>Philadelphia 76ers</t>
@@ -14476,12 +14468,8 @@
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr"/>
       <c r="H159" t="inlineStr"/>
-      <c r="I159" t="n">
-        <v>0.3272</v>
-      </c>
-      <c r="J159" t="n">
-        <v>0.6728</v>
-      </c>
+      <c r="I159" t="inlineStr"/>
+      <c r="J159" t="inlineStr"/>
       <c r="K159" t="inlineStr">
         <is>
           <t>Minnesota Timberwolves</t>
@@ -14523,12 +14511,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-05-01T23:00:00+00:00</t>
+          <t>2026-05-01T04:00:00+00:00</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2026-05-02 07:00:00</t>
+          <t>2026-05-01 12:00:00</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -14607,12 +14595,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-05-01T23:00:00+00:00</t>
+          <t>2026-05-01T04:00:00+00:00</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2026-05-02 07:00:00</t>
+          <t>2026-05-01 12:00:00</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -14671,12 +14659,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-05-01T23:30:00+00:00</t>
+          <t>2026-05-01T04:00:00+00:00</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2026-05-02 07:30:00</t>
+          <t>2026-05-01 12:00:00</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -15148,12 +15136,8 @@
       <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr"/>
       <c r="H169" t="inlineStr"/>
-      <c r="I169" t="n">
-        <v>0.5935</v>
-      </c>
-      <c r="J169" t="n">
-        <v>0.4065</v>
-      </c>
+      <c r="I169" t="inlineStr"/>
+      <c r="J169" t="inlineStr"/>
       <c r="K169" t="inlineStr">
         <is>
           <t>Los Angeles Lakers</t>
@@ -15182,7 +15166,7 @@
       </c>
       <c r="AA169" t="inlineStr">
         <is>
-          <t>https://polymarket.com/event/nba-lal-hou-2026-05-01</t>
+          <t>https://polymarket.com/event/nba-hou-lal-2026-04-29</t>
         </is>
       </c>
       <c r="AB169" t="inlineStr"/>
@@ -15434,7 +15418,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -15528,7 +15512,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -15622,7 +15606,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -15716,7 +15700,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -15810,7 +15794,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -15912,7 +15896,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -16014,7 +15998,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -16116,7 +16100,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -16218,7 +16202,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -16324,7 +16308,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -16426,7 +16410,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -16532,7 +16516,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -16634,7 +16618,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -16740,7 +16724,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -16842,7 +16826,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -16948,7 +16932,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -17050,7 +17034,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -17148,7 +17132,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -17246,7 +17230,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -17340,7 +17324,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -17442,7 +17426,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -17544,7 +17528,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -17646,7 +17630,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -17748,7 +17732,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -17846,7 +17830,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -17944,7 +17928,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -18042,7 +18026,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -18140,7 +18124,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -18238,7 +18222,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -18336,7 +18320,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -18438,7 +18422,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -18540,7 +18524,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -18642,7 +18626,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -18744,7 +18728,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -18842,7 +18826,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -18940,7 +18924,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -19038,7 +19022,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -19140,7 +19124,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -19242,7 +19226,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -19344,7 +19328,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -19446,7 +19430,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -19548,7 +19532,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -19654,7 +19638,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -19756,7 +19740,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -19858,7 +19842,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -19942,7 +19926,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -20026,7 +20010,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -20110,7 +20094,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -20194,7 +20178,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -20296,7 +20280,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -20390,7 +20374,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -20496,7 +20480,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -20602,7 +20586,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -20708,7 +20692,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -20814,7 +20798,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -20916,7 +20900,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -21018,7 +21002,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -21120,7 +21104,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -21222,7 +21206,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -21328,7 +21312,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -21434,7 +21418,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -21540,7 +21524,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -21650,7 +21634,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -21752,7 +21736,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -21854,7 +21838,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -21952,7 +21936,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -22054,7 +22038,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -22156,7 +22140,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -22258,7 +22242,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
@@ -22342,7 +22326,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -22436,7 +22420,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -22542,7 +22526,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -22640,7 +22624,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -22746,7 +22730,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -22848,7 +22832,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -22950,7 +22934,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -23054,7 +23038,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -23158,7 +23142,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -23258,7 +23242,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -23362,7 +23346,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -23466,7 +23450,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -23570,7 +23554,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -23670,7 +23654,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -23774,7 +23758,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -23878,7 +23862,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -23982,7 +23966,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -24082,7 +24066,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -24182,7 +24166,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -24278,7 +24262,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -24374,7 +24358,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -24478,7 +24462,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -24582,7 +24566,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -24662,7 +24646,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -24750,7 +24734,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -24822,7 +24806,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -24894,7 +24878,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -24966,7 +24950,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -25050,7 +25034,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -25122,7 +25106,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -25206,7 +25190,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -25278,7 +25262,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -25350,7 +25334,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -25422,7 +25406,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -25494,7 +25478,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -25566,7 +25550,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -25634,7 +25618,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -25702,7 +25686,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
@@ -25774,7 +25758,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
@@ -25846,7 +25830,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
@@ -25918,7 +25902,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
@@ -25990,7 +25974,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
@@ -26062,7 +26046,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
@@ -26134,7 +26118,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -26206,7 +26190,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -26278,7 +26262,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -26350,7 +26334,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -26422,7 +26406,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -26494,7 +26478,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -26566,7 +26550,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
@@ -26638,7 +26622,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F121" t="inlineStr"/>
@@ -26710,7 +26694,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
@@ -26782,7 +26766,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F123" t="inlineStr"/>
@@ -26854,7 +26838,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
@@ -26926,7 +26910,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -26998,7 +26982,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -27070,7 +27054,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
@@ -27138,7 +27122,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F128" t="inlineStr"/>
@@ -27210,7 +27194,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F129" t="inlineStr"/>
@@ -27278,7 +27262,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
@@ -27346,7 +27330,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F131" t="inlineStr"/>
@@ -27414,7 +27398,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F132" t="inlineStr"/>
@@ -27482,7 +27466,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F133" t="inlineStr"/>
@@ -27550,7 +27534,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F134" t="inlineStr"/>
@@ -27618,7 +27602,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F135" t="inlineStr"/>
@@ -27690,7 +27674,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F136" t="inlineStr"/>
@@ -27762,7 +27746,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F137" t="inlineStr"/>
@@ -27834,7 +27818,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F138" t="inlineStr"/>
@@ -27906,7 +27890,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
@@ -27978,7 +27962,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F140" t="inlineStr"/>
@@ -28050,7 +28034,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F141" t="inlineStr"/>
@@ -28122,7 +28106,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F142" t="inlineStr"/>
@@ -28194,7 +28178,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F143" t="inlineStr"/>
@@ -28266,7 +28250,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F144" t="inlineStr"/>
@@ -28338,7 +28322,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F145" t="inlineStr"/>
@@ -28410,7 +28394,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F146" t="inlineStr"/>
@@ -28478,7 +28462,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F147" t="inlineStr"/>
@@ -28546,7 +28530,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F148" t="inlineStr"/>
@@ -28618,7 +28602,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F149" t="inlineStr"/>
@@ -28690,7 +28674,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F150" t="inlineStr"/>
@@ -28762,7 +28746,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F151" t="inlineStr"/>
@@ -28834,7 +28818,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F152" t="inlineStr"/>
@@ -28906,7 +28890,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F153" t="inlineStr"/>
@@ -28978,7 +28962,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F154" t="inlineStr"/>
@@ -29050,7 +29034,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>in_play</t>
         </is>
       </c>
       <c r="F155" t="inlineStr"/>
@@ -29107,12 +29091,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-05-01T23:00:00+00:00</t>
+          <t>2026-05-01T04:00:00+00:00</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2026-05-02 07:00:00</t>
+          <t>2026-05-01 12:00:00</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">

</xml_diff>

<commit_message>
Preserve historical settled winners without db
</commit_message>
<xml_diff>
--- a/backtest.xlsx
+++ b/backtest.xlsx
@@ -13778,7 +13778,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>in_play</t>
+          <t>final</t>
         </is>
       </c>
       <c r="F155" t="inlineStr"/>
@@ -14178,7 +14178,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>final</t>
         </is>
       </c>
       <c r="F161" t="inlineStr"/>
@@ -28198,7 +28198,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>in_play</t>
+          <t>final</t>
         </is>
       </c>
       <c r="F155" t="inlineStr"/>
@@ -28342,7 +28342,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>final</t>
         </is>
       </c>
       <c r="F157" t="inlineStr"/>

</xml_diff>